<commit_message>
feat: update data files and config for March 2026 progress
</commit_message>
<xml_diff>
--- a/Data_thang/Thang_03_2026.xlsx
+++ b/Data_thang/Thang_03_2026.xlsx
@@ -7265,17 +7265,17 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Trực</t>
         </is>
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/03/2026 09:37:23</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr">
@@ -7293,7 +7293,7 @@
       </c>
       <c r="J5" s="11" t="inlineStr">
         <is>
-          <t>kythuat</t>
+          <t>lanhn</t>
         </is>
       </c>
     </row>
@@ -8225,17 +8225,17 @@
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>H.Trang</t>
         </is>
       </c>
       <c r="E25" s="16" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/03/2026 10:04:16</t>
         </is>
       </c>
       <c r="G25" s="12" t="inlineStr">
@@ -8513,17 +8513,17 @@
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Gia Thư</t>
         </is>
       </c>
       <c r="E31" s="16" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/03/2026 11:42:17</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
@@ -8541,7 +8541,7 @@
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>kythuat</t>
+          <t>lanhn</t>
         </is>
       </c>
     </row>
@@ -18726,17 +18726,17 @@
       </c>
       <c r="D243" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Gia Thư</t>
         </is>
       </c>
       <c r="E243" s="16" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="F243" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/03/2026 09:13:06</t>
         </is>
       </c>
       <c r="G243" s="12" t="inlineStr">

</xml_diff>